<commit_message>
feat: sync user auth, remove Analisa Lain, unify filter box and fix category mapping for TOKEN PLN & GAME
</commit_message>
<xml_diff>
--- a/pages/sco/KPI_SCO.xlsx
+++ b/pages/sco/KPI_SCO.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WEB REPORT\pages\sco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DC2FDC-C10D-40EE-98FD-56AD70D615B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB56389F-C1F3-43AA-BAAF-B8169C01C92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_SCO" sheetId="2" r:id="rId1"/>
     <sheet name="KPI_DSO" sheetId="3" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">KPI_SCO!$A$1:$Q$52</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
@@ -482,6 +485,36 @@
     <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -525,36 +558,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -30860,69 +30863,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="39">
+      <c r="B1" s="24">
         <v>0.3</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="42">
+      <c r="C1" s="25"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="27">
         <v>0.2</v>
       </c>
-      <c r="F1" s="43"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="45">
+      <c r="F1" s="28"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="30">
         <v>0.3</v>
       </c>
-      <c r="I1" s="46"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="45">
+      <c r="I1" s="31"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="30">
         <v>0.2</v>
       </c>
-      <c r="L1" s="46"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="36" t="s">
+      <c r="L1" s="31"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="46" t="s">
         <v>24</v>
       </c>
       <c r="O1" s="12"/>
-      <c r="P1" s="23" t="s">
+      <c r="P1" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="26" t="s">
+      <c r="Q1" s="36" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="38"/>
-      <c r="B2" s="27" t="s">
+      <c r="A2" s="23"/>
+      <c r="B2" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="33" t="s">
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="34"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="33" t="s">
+      <c r="I2" s="44"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="34"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="37"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="47"/>
       <c r="O2" s="12"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="26"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="36"/>
     </row>
     <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="38"/>
+      <c r="A3" s="23"/>
       <c r="B3" s="13" t="s">
         <v>31</v>
       </c>
@@ -30959,10 +30962,10 @@
       <c r="M3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="37"/>
+      <c r="N3" s="47"/>
       <c r="O3" s="12"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="26"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="36"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="16">
@@ -31666,11 +31669,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
     <mergeCell ref="P1:P3"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="B2:D2"/>
@@ -31678,6 +31676,11 @@
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="N1:N3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D15 G4:G15 J4:J15 M4:N15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>